<commit_message>
funcionando e publicado para novo outlook
</commit_message>
<xml_diff>
--- a/testes/teste1.xlsx
+++ b/testes/teste1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJETOS\Innova_ExcelVerifier\testes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7757186A-CD6C-4303-B404-C65F55D15A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C3B94B3-D710-40CA-9CA3-2906EE16FDC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="21600" windowHeight="12670" tabRatio="833" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51105" yWindow="120" windowWidth="21600" windowHeight="11715" tabRatio="833" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMO" sheetId="3" r:id="rId1"/>
@@ -1499,7 +1499,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="135">
   <si>
     <t xml:space="preserve">PLANILHA DE ESTIMATIVA DE CUSTOS </t>
   </si>
@@ -2503,9 +2503,6 @@
   </si>
   <si>
     <t>teste</t>
-  </si>
-  <si>
-    <t>etstete</t>
   </si>
 </sst>
 </file>
@@ -4457,58 +4454,17 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="14" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="14" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="10" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="23" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="23" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="16" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4549,11 +4505,52 @@
     <xf numFmtId="49" fontId="10" fillId="10" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="10" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="13" fillId="13" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="16" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="25" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="25" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="14" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="14" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="18" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -5237,7 +5234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q781"/>
+  <dimension ref="A1:P781"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.453125" style="1" customWidth="1"/>
@@ -5253,26 +5250,14 @@
     <col min="14" max="16384" width="14.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B1" s="24"/>
       <c r="C1" s="23"/>
       <c r="D1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B2" s="21"/>
       <c r="C2" s="20" t="s">
         <v>1</v>
@@ -5280,20 +5265,8 @@
       <c r="D2" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="N2" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="21"/>
       <c r="C3" s="20" t="s">
         <v>2</v>
@@ -5301,11 +5274,8 @@
       <c r="D3" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B4" s="21"/>
       <c r="C4" s="20" t="s">
         <v>3</v>
@@ -5313,11 +5283,8 @@
       <c r="D4" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B5" s="21"/>
       <c r="C5" s="20" t="s">
         <v>4</v>
@@ -5326,7 +5293,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B6" s="21"/>
       <c r="C6" s="20" t="s">
         <v>5</v>
@@ -5335,7 +5302,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B7" s="21"/>
       <c r="C7" s="20" t="s">
         <v>6</v>
@@ -5344,7 +5311,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B8" s="21"/>
       <c r="C8" s="20" t="s">
         <v>7</v>
@@ -5353,7 +5320,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B9" s="21"/>
       <c r="C9" s="20" t="s">
         <v>55</v>
@@ -5362,7 +5329,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B10" s="21"/>
       <c r="C10" s="20" t="s">
         <v>54</v>
@@ -5371,7 +5338,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B11" s="21"/>
       <c r="C11" s="20" t="s">
         <v>103</v>
@@ -5380,12 +5347,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="19"/>
       <c r="C12" s="18"/>
       <c r="D12" s="28"/>
     </row>
-    <row r="13" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="17"/>
@@ -5399,7 +5366,7 @@
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="17"/>
@@ -5423,7 +5390,7 @@
       </c>
       <c r="P14" s="223"/>
     </row>
-    <row r="15" spans="1:17" s="5" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" s="5" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="8"/>
       <c r="B15" s="228" t="s">
         <v>52</v>
@@ -5449,7 +5416,7 @@
       </c>
       <c r="P15" s="225"/>
     </row>
-    <row r="16" spans="1:17" s="5" customFormat="1" ht="31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" s="5" customFormat="1" ht="31" x14ac:dyDescent="0.35">
       <c r="A16" s="8"/>
       <c r="B16" s="233" t="s">
         <v>50</v>
@@ -8218,13 +8185,13 @@
         <f>RESUMO!D8</f>
         <v>BO_0001_26</v>
       </c>
-      <c r="K9" s="245"/>
-      <c r="L9" s="245"/>
+      <c r="K9" s="264"/>
+      <c r="L9" s="264"/>
       <c r="M9" s="37"/>
       <c r="N9" s="38"/>
       <c r="O9" s="37"/>
-      <c r="P9" s="245"/>
-      <c r="Q9" s="245"/>
+      <c r="P9" s="264"/>
+      <c r="Q9" s="264"/>
       <c r="R9" s="68"/>
       <c r="S9" s="37"/>
       <c r="T9" s="37"/>
@@ -8307,10 +8274,10 @@
       <c r="S11" s="71"/>
       <c r="T11" s="37"/>
       <c r="U11" s="39"/>
-      <c r="V11" s="252" t="s">
+      <c r="V11" s="266" t="s">
         <v>96</v>
       </c>
-      <c r="W11" s="253"/>
+      <c r="W11" s="267"/>
       <c r="Z11" s="37"/>
       <c r="AA11" s="37"/>
       <c r="AE11" s="37"/>
@@ -8345,10 +8312,10 @@
       <c r="S12" s="71"/>
       <c r="T12" s="37"/>
       <c r="U12" s="39"/>
-      <c r="V12" s="252" t="s">
+      <c r="V12" s="266" t="s">
         <v>96</v>
       </c>
-      <c r="W12" s="253"/>
+      <c r="W12" s="267"/>
       <c r="Z12" s="37"/>
       <c r="AA12" s="37"/>
       <c r="AE12" s="37"/>
@@ -8450,46 +8417,46 @@
       <c r="I15" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="K15" s="243" t="s">
+      <c r="K15" s="272" t="s">
         <v>15</v>
       </c>
-      <c r="L15" s="244"/>
+      <c r="L15" s="273"/>
       <c r="M15" s="92"/>
       <c r="N15" s="75"/>
       <c r="O15" s="92"/>
-      <c r="P15" s="251" t="s">
+      <c r="P15" s="265" t="s">
         <v>80</v>
       </c>
-      <c r="Q15" s="251"/>
-      <c r="R15" s="251"/>
+      <c r="Q15" s="265"/>
+      <c r="R15" s="265"/>
       <c r="S15" s="92"/>
-      <c r="T15" s="246" t="s">
+      <c r="T15" s="261" t="s">
         <v>40</v>
       </c>
-      <c r="U15" s="247"/>
-      <c r="V15" s="247"/>
-      <c r="W15" s="247"/>
-      <c r="X15" s="247"/>
-      <c r="Y15" s="247"/>
-      <c r="Z15" s="247"/>
-      <c r="AA15" s="248"/>
-      <c r="AC15" s="246" t="s">
+      <c r="U15" s="262"/>
+      <c r="V15" s="262"/>
+      <c r="W15" s="262"/>
+      <c r="X15" s="262"/>
+      <c r="Y15" s="262"/>
+      <c r="Z15" s="262"/>
+      <c r="AA15" s="263"/>
+      <c r="AC15" s="261" t="s">
         <v>43</v>
       </c>
-      <c r="AD15" s="247"/>
-      <c r="AE15" s="247"/>
-      <c r="AF15" s="247"/>
-      <c r="AG15" s="247"/>
-      <c r="AH15" s="247"/>
-      <c r="AI15" s="247"/>
-      <c r="AJ15" s="247"/>
-      <c r="AK15" s="247"/>
-      <c r="AL15" s="247"/>
-      <c r="AM15" s="247"/>
-      <c r="AN15" s="247"/>
-      <c r="AO15" s="247"/>
-      <c r="AP15" s="247"/>
-      <c r="AQ15" s="248"/>
+      <c r="AD15" s="262"/>
+      <c r="AE15" s="262"/>
+      <c r="AF15" s="262"/>
+      <c r="AG15" s="262"/>
+      <c r="AH15" s="262"/>
+      <c r="AI15" s="262"/>
+      <c r="AJ15" s="262"/>
+      <c r="AK15" s="262"/>
+      <c r="AL15" s="262"/>
+      <c r="AM15" s="262"/>
+      <c r="AN15" s="262"/>
+      <c r="AO15" s="262"/>
+      <c r="AP15" s="262"/>
+      <c r="AQ15" s="263"/>
     </row>
     <row r="16" spans="2:43" ht="51" x14ac:dyDescent="0.4">
       <c r="B16" s="93">
@@ -8539,10 +8506,10 @@
       <c r="W16" s="101" t="s">
         <v>24</v>
       </c>
-      <c r="X16" s="249" t="s">
+      <c r="X16" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="Y16" s="250"/>
+      <c r="Y16" s="240"/>
       <c r="Z16" s="102" t="s">
         <v>25</v>
       </c>
@@ -8579,10 +8546,10 @@
       <c r="AL16" s="103" t="s">
         <v>41</v>
       </c>
-      <c r="AM16" s="249" t="s">
+      <c r="AM16" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="AN16" s="250"/>
+      <c r="AN16" s="240"/>
       <c r="AO16" s="103" t="s">
         <v>19</v>
       </c>
@@ -8867,10 +8834,10 @@
       <c r="W19" s="101" t="s">
         <v>24</v>
       </c>
-      <c r="X19" s="249" t="s">
+      <c r="X19" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="Y19" s="250"/>
+      <c r="Y19" s="240"/>
       <c r="Z19" s="102" t="s">
         <v>25</v>
       </c>
@@ -8907,10 +8874,10 @@
       <c r="AL19" s="103" t="s">
         <v>41</v>
       </c>
-      <c r="AM19" s="249" t="s">
+      <c r="AM19" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="AN19" s="250"/>
+      <c r="AN19" s="240"/>
       <c r="AO19" s="103" t="s">
         <v>19</v>
       </c>
@@ -9201,10 +9168,10 @@
       <c r="W22" s="101" t="s">
         <v>24</v>
       </c>
-      <c r="X22" s="249" t="s">
+      <c r="X22" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="Y22" s="250"/>
+      <c r="Y22" s="240"/>
       <c r="Z22" s="102" t="s">
         <v>25</v>
       </c>
@@ -9241,10 +9208,10 @@
       <c r="AL22" s="103" t="s">
         <v>41</v>
       </c>
-      <c r="AM22" s="249" t="s">
+      <c r="AM22" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="AN22" s="250"/>
+      <c r="AN22" s="240"/>
       <c r="AO22" s="103" t="s">
         <v>19</v>
       </c>
@@ -9640,10 +9607,10 @@
       <c r="W26" s="101" t="s">
         <v>24</v>
       </c>
-      <c r="X26" s="249" t="s">
+      <c r="X26" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="Y26" s="250"/>
+      <c r="Y26" s="240"/>
       <c r="Z26" s="102" t="s">
         <v>25</v>
       </c>
@@ -9680,10 +9647,10 @@
       <c r="AL26" s="103" t="s">
         <v>41</v>
       </c>
-      <c r="AM26" s="249" t="s">
+      <c r="AM26" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="AN26" s="250"/>
+      <c r="AN26" s="240"/>
       <c r="AO26" s="103" t="s">
         <v>19</v>
       </c>
@@ -10352,10 +10319,10 @@
       <c r="W33" s="101" t="s">
         <v>24</v>
       </c>
-      <c r="X33" s="249" t="s">
+      <c r="X33" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="Y33" s="250"/>
+      <c r="Y33" s="240"/>
       <c r="Z33" s="102" t="s">
         <v>25</v>
       </c>
@@ -10392,10 +10359,10 @@
       <c r="AL33" s="103" t="s">
         <v>41</v>
       </c>
-      <c r="AM33" s="249" t="s">
+      <c r="AM33" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="AN33" s="250"/>
+      <c r="AN33" s="240"/>
       <c r="AO33" s="103" t="s">
         <v>19</v>
       </c>
@@ -10560,10 +10527,10 @@
       <c r="W35" s="160" t="s">
         <v>24</v>
       </c>
-      <c r="X35" s="249" t="s">
+      <c r="X35" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="Y35" s="250"/>
+      <c r="Y35" s="240"/>
       <c r="Z35" s="161" t="s">
         <v>25</v>
       </c>
@@ -10590,24 +10557,24 @@
       </c>
       <c r="AK35" s="103"/>
       <c r="AL35" s="103"/>
-      <c r="AM35" s="249" t="s">
+      <c r="AM35" s="239" t="s">
         <v>42</v>
       </c>
-      <c r="AN35" s="250"/>
+      <c r="AN35" s="240"/>
       <c r="AO35" s="103"/>
       <c r="AP35" s="103"/>
       <c r="AQ35" s="103"/>
     </row>
     <row r="36" spans="2:43" ht="27.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="269" t="s">
+      <c r="B36" s="254" t="s">
         <v>65</v>
       </c>
-      <c r="C36" s="270"/>
-      <c r="D36" s="270"/>
-      <c r="E36" s="270"/>
-      <c r="F36" s="270"/>
-      <c r="G36" s="270"/>
-      <c r="H36" s="270"/>
+      <c r="C36" s="255"/>
+      <c r="D36" s="255"/>
+      <c r="E36" s="255"/>
+      <c r="F36" s="255"/>
+      <c r="G36" s="255"/>
+      <c r="H36" s="255"/>
       <c r="I36" s="162">
         <f>SUMIF(D:D,"( I )",H:H)</f>
         <v>75600</v>
@@ -10675,15 +10642,15 @@
       <c r="AQ36" s="35"/>
     </row>
     <row r="37" spans="2:43" ht="27.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="241" t="s">
+      <c r="B37" s="256" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="242"/>
-      <c r="D37" s="242"/>
-      <c r="E37" s="242"/>
-      <c r="F37" s="242"/>
-      <c r="G37" s="242"/>
-      <c r="H37" s="242"/>
+      <c r="C37" s="257"/>
+      <c r="D37" s="257"/>
+      <c r="E37" s="257"/>
+      <c r="F37" s="257"/>
+      <c r="G37" s="257"/>
+      <c r="H37" s="257"/>
       <c r="I37" s="171">
         <f>SUMIF(D:D,"( T )",H:H)</f>
         <v>0</v>
@@ -10701,7 +10668,7 @@
       <c r="U37" s="172"/>
       <c r="V37" s="165"/>
       <c r="W37" s="165"/>
-      <c r="Z37" s="260" t="s">
+      <c r="Z37" s="245" t="s">
         <v>97</v>
       </c>
       <c r="AB37" s="41"/>
@@ -10713,15 +10680,15 @@
       <c r="AQ37" s="35"/>
     </row>
     <row r="38" spans="2:43" ht="27.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B38" s="241" t="s">
+      <c r="B38" s="256" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="242"/>
-      <c r="D38" s="242"/>
-      <c r="E38" s="242"/>
-      <c r="F38" s="242"/>
-      <c r="G38" s="242"/>
-      <c r="H38" s="242"/>
+      <c r="C38" s="257"/>
+      <c r="D38" s="257"/>
+      <c r="E38" s="257"/>
+      <c r="F38" s="257"/>
+      <c r="G38" s="257"/>
+      <c r="H38" s="257"/>
       <c r="I38" s="173">
         <f>SUMIF(D:D,"( C )",H:H)</f>
         <v>0</v>
@@ -10739,7 +10706,7 @@
       <c r="U38" s="172"/>
       <c r="V38" s="165"/>
       <c r="W38" s="165"/>
-      <c r="Z38" s="261"/>
+      <c r="Z38" s="246"/>
       <c r="AB38" s="41"/>
       <c r="AD38" s="74"/>
       <c r="AF38" s="35"/>
@@ -10749,15 +10716,15 @@
       <c r="AQ38" s="35"/>
     </row>
     <row r="39" spans="2:43" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B39" s="271" t="s">
+      <c r="B39" s="258" t="s">
         <v>94</v>
       </c>
-      <c r="C39" s="272"/>
-      <c r="D39" s="272"/>
-      <c r="E39" s="272"/>
-      <c r="F39" s="272"/>
-      <c r="G39" s="272"/>
-      <c r="H39" s="273"/>
+      <c r="C39" s="259"/>
+      <c r="D39" s="259"/>
+      <c r="E39" s="259"/>
+      <c r="F39" s="259"/>
+      <c r="G39" s="259"/>
+      <c r="H39" s="260"/>
       <c r="I39" s="174">
         <f>SUM(I36:I38)</f>
         <v>75600</v>
@@ -10776,20 +10743,20 @@
       <c r="Q39" s="164"/>
       <c r="R39" s="164"/>
       <c r="S39" s="131"/>
-      <c r="T39" s="256" t="s">
+      <c r="T39" s="241" t="s">
         <v>37</v>
       </c>
-      <c r="U39" s="257"/>
+      <c r="U39" s="242"/>
       <c r="V39" s="177"/>
       <c r="W39" s="178">
         <f>SUM(AA36+I40+I41)</f>
         <v>14620</v>
       </c>
       <c r="AB39" s="41"/>
-      <c r="AD39" s="258" t="s">
+      <c r="AD39" s="243" t="s">
         <v>37</v>
       </c>
-      <c r="AE39" s="259"/>
+      <c r="AE39" s="244"/>
       <c r="AF39" s="179" t="e">
         <f>SUM(AN36+AI36+I40+I41)</f>
         <v>#VALUE!</v>
@@ -10800,14 +10767,14 @@
       <c r="AQ39" s="35"/>
     </row>
     <row r="40" spans="2:43" ht="27.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B40" s="237" t="s">
+      <c r="B40" s="268" t="s">
         <v>125</v>
       </c>
-      <c r="C40" s="238"/>
-      <c r="D40" s="238"/>
-      <c r="E40" s="238"/>
-      <c r="F40" s="238"/>
-      <c r="G40" s="238"/>
+      <c r="C40" s="269"/>
+      <c r="D40" s="269"/>
+      <c r="E40" s="269"/>
+      <c r="F40" s="269"/>
+      <c r="G40" s="269"/>
       <c r="H40" s="180">
         <v>0</v>
       </c>
@@ -10853,14 +10820,14 @@
       <c r="AQ40" s="35"/>
     </row>
     <row r="41" spans="2:43" ht="27.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B41" s="239" t="s">
+      <c r="B41" s="270" t="s">
         <v>59</v>
       </c>
-      <c r="C41" s="240"/>
-      <c r="D41" s="240"/>
-      <c r="E41" s="240"/>
-      <c r="F41" s="240"/>
-      <c r="G41" s="240"/>
+      <c r="C41" s="271"/>
+      <c r="D41" s="271"/>
+      <c r="E41" s="271"/>
+      <c r="F41" s="271"/>
+      <c r="G41" s="271"/>
       <c r="H41" s="191">
         <v>0.1</v>
       </c>
@@ -10895,14 +10862,14 @@
       <c r="AQ41" s="35"/>
     </row>
     <row r="42" spans="2:43" ht="27.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B42" s="262" t="s">
+      <c r="B42" s="247" t="s">
         <v>100</v>
       </c>
-      <c r="C42" s="263"/>
-      <c r="D42" s="263"/>
-      <c r="E42" s="263"/>
-      <c r="F42" s="263"/>
-      <c r="G42" s="263"/>
+      <c r="C42" s="248"/>
+      <c r="D42" s="248"/>
+      <c r="E42" s="248"/>
+      <c r="F42" s="248"/>
+      <c r="G42" s="248"/>
       <c r="H42" s="197" t="s">
         <v>57</v>
       </c>
@@ -10947,15 +10914,15 @@
       <c r="AQ42" s="35"/>
     </row>
     <row r="43" spans="2:43" ht="28.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B43" s="264" t="s">
+      <c r="B43" s="249" t="s">
         <v>39</v>
       </c>
-      <c r="C43" s="265"/>
-      <c r="D43" s="265"/>
-      <c r="E43" s="265"/>
-      <c r="F43" s="265"/>
-      <c r="G43" s="265"/>
-      <c r="H43" s="266"/>
+      <c r="C43" s="250"/>
+      <c r="D43" s="250"/>
+      <c r="E43" s="250"/>
+      <c r="F43" s="250"/>
+      <c r="G43" s="250"/>
+      <c r="H43" s="251"/>
       <c r="I43" s="202">
         <f>SUM(I39:I42)</f>
         <v>99000</v>
@@ -11006,11 +10973,11 @@
       <c r="G44" s="33"/>
       <c r="H44" s="33"/>
       <c r="I44" s="34"/>
-      <c r="K44" s="267">
+      <c r="K44" s="252">
         <f>SUM(K43:L43)</f>
         <v>99000</v>
       </c>
-      <c r="L44" s="268"/>
+      <c r="L44" s="253"/>
       <c r="M44" s="131"/>
       <c r="N44" s="72"/>
       <c r="O44" s="131"/>
@@ -11026,15 +10993,15 @@
       <c r="AQ44" s="35"/>
     </row>
     <row r="45" spans="2:43" x14ac:dyDescent="0.4">
-      <c r="B45" s="254" t="s">
+      <c r="B45" s="237" t="s">
         <v>98</v>
       </c>
-      <c r="C45" s="254"/>
-      <c r="D45" s="254"/>
-      <c r="E45" s="254"/>
-      <c r="F45" s="254"/>
-      <c r="G45" s="254"/>
-      <c r="H45" s="254"/>
+      <c r="C45" s="237"/>
+      <c r="D45" s="237"/>
+      <c r="E45" s="237"/>
+      <c r="F45" s="237"/>
+      <c r="G45" s="237"/>
+      <c r="H45" s="237"/>
       <c r="I45" s="208"/>
       <c r="K45" s="209"/>
       <c r="L45" s="210"/>
@@ -11059,15 +11026,15 @@
       <c r="AQ45" s="35"/>
     </row>
     <row r="46" spans="2:43" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="238" t="s">
         <v>99</v>
       </c>
-      <c r="C46" s="255"/>
-      <c r="D46" s="255"/>
-      <c r="E46" s="255"/>
-      <c r="F46" s="255"/>
-      <c r="G46" s="255"/>
-      <c r="H46" s="255"/>
+      <c r="C46" s="238"/>
+      <c r="D46" s="238"/>
+      <c r="E46" s="238"/>
+      <c r="F46" s="238"/>
+      <c r="G46" s="238"/>
+      <c r="H46" s="238"/>
       <c r="I46" s="213"/>
       <c r="K46" s="214"/>
       <c r="L46" s="215"/>
@@ -11092,15 +11059,15 @@
       <c r="AQ46" s="207"/>
     </row>
     <row r="47" spans="2:43" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="254" t="s">
+      <c r="B47" s="237" t="s">
         <v>112</v>
       </c>
-      <c r="C47" s="254"/>
-      <c r="D47" s="254"/>
-      <c r="E47" s="254"/>
-      <c r="F47" s="254"/>
-      <c r="G47" s="254"/>
-      <c r="H47" s="254"/>
+      <c r="C47" s="237"/>
+      <c r="D47" s="237"/>
+      <c r="E47" s="237"/>
+      <c r="F47" s="237"/>
+      <c r="G47" s="237"/>
+      <c r="H47" s="237"/>
       <c r="I47" s="208"/>
       <c r="AE47" s="211" t="s">
         <v>89</v>
@@ -11158,6 +11125,25 @@
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B38:H38"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="T15:AA15"/>
+    <mergeCell ref="AC15:AQ15"/>
+    <mergeCell ref="AM16:AN16"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="P15:R15"/>
+    <mergeCell ref="V11:W11"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="AM19:AN19"/>
+    <mergeCell ref="X16:Y16"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="X22:Y22"/>
+    <mergeCell ref="X26:Y26"/>
+    <mergeCell ref="AM22:AN22"/>
+    <mergeCell ref="AM26:AN26"/>
     <mergeCell ref="B45:H45"/>
     <mergeCell ref="B46:H46"/>
     <mergeCell ref="B47:H47"/>
@@ -11174,25 +11160,6 @@
     <mergeCell ref="B36:H36"/>
     <mergeCell ref="B37:H37"/>
     <mergeCell ref="B39:H39"/>
-    <mergeCell ref="AM19:AN19"/>
-    <mergeCell ref="X16:Y16"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="X22:Y22"/>
-    <mergeCell ref="X26:Y26"/>
-    <mergeCell ref="AM22:AN22"/>
-    <mergeCell ref="AM26:AN26"/>
-    <mergeCell ref="T15:AA15"/>
-    <mergeCell ref="AC15:AQ15"/>
-    <mergeCell ref="AM16:AN16"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="P15:R15"/>
-    <mergeCell ref="V11:W11"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="B40:G40"/>
-    <mergeCell ref="B41:G41"/>
-    <mergeCell ref="B38:H38"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="K9:L9"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="AC17:AC18 AC21 AC23:AC25 AC27 AC30 AC32 AC34">

</xml_diff>